<commit_message>
Atualização de comentários no código
</commit_message>
<xml_diff>
--- a/backend/arq/search_albums_scorpion.xlsx
+++ b/backend/arq/search_albums_scorpion.xlsx
@@ -67,27 +67,27 @@
     <t>https://api.spotify.com/v1/albums/6ZWL1xSTEvqs5A6dBh8vZw</t>
   </si>
   <si>
+    <t>https://api.spotify.com/v1/albums/2epkTConsXtPOHY9QhvqeR</t>
+  </si>
+  <si>
     <t>https://api.spotify.com/v1/albums/71cfSO0iO1fjgQLEb3Wc6C</t>
   </si>
   <si>
+    <t>https://api.spotify.com/v1/albums/7aIgGWlHdcPXOfONtXVliK</t>
+  </si>
+  <si>
+    <t>https://api.spotify.com/v1/albums/6x75r5C54z1quun86Bbqbr</t>
+  </si>
+  <si>
+    <t>https://api.spotify.com/v1/albums/5z5s71RoLOhdB8SwPfru0I</t>
+  </si>
+  <si>
     <t>https://api.spotify.com/v1/albums/4vQ96yyyYbaeTQujH3iTtd</t>
   </si>
   <si>
-    <t>https://api.spotify.com/v1/albums/2epkTConsXtPOHY9QhvqeR</t>
-  </si>
-  <si>
-    <t>https://api.spotify.com/v1/albums/6x75r5C54z1quun86Bbqbr</t>
-  </si>
-  <si>
     <t>https://api.spotify.com/v1/albums/3dLKM8bD8R3H3XnSOXGjTF</t>
   </si>
   <si>
-    <t>https://api.spotify.com/v1/albums/7aIgGWlHdcPXOfONtXVliK</t>
-  </si>
-  <si>
-    <t>https://api.spotify.com/v1/albums/5z5s71RoLOhdB8SwPfru0I</t>
-  </si>
-  <si>
     <t>1ATL5GLyefJaxhQzSPVrLX</t>
   </si>
   <si>
@@ -97,27 +97,27 @@
     <t>6ZWL1xSTEvqs5A6dBh8vZw</t>
   </si>
   <si>
+    <t>2epkTConsXtPOHY9QhvqeR</t>
+  </si>
+  <si>
     <t>71cfSO0iO1fjgQLEb3Wc6C</t>
   </si>
   <si>
+    <t>7aIgGWlHdcPXOfONtXVliK</t>
+  </si>
+  <si>
+    <t>6x75r5C54z1quun86Bbqbr</t>
+  </si>
+  <si>
+    <t>5z5s71RoLOhdB8SwPfru0I</t>
+  </si>
+  <si>
     <t>4vQ96yyyYbaeTQujH3iTtd</t>
   </si>
   <si>
-    <t>2epkTConsXtPOHY9QhvqeR</t>
-  </si>
-  <si>
-    <t>6x75r5C54z1quun86Bbqbr</t>
-  </si>
-  <si>
     <t>3dLKM8bD8R3H3XnSOXGjTF</t>
   </si>
   <si>
-    <t>7aIgGWlHdcPXOfONtXVliK</t>
-  </si>
-  <si>
-    <t>5z5s71RoLOhdB8SwPfru0I</t>
-  </si>
-  <si>
     <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273f907de96b9a4fbc04accc0d5', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02f907de96b9a4fbc04accc0d5', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851f907de96b9a4fbc04accc0d5', 'width': 64}]</t>
   </si>
   <si>
@@ -127,27 +127,27 @@
     <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b2730a825fea8b9095572e5130ef', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e020a825fea8b9095572e5130ef', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d000048510a825fea8b9095572e5130ef', 'width': 64}]</t>
   </si>
   <si>
+    <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b2732dd8a31709137799f5c937f2', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e022dd8a31709137799f5c937f2', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d000048512dd8a31709137799f5c937f2', 'width': 64}]</t>
+  </si>
+  <si>
     <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273926764eed4da16a86b9ce33e', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02926764eed4da16a86b9ce33e', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851926764eed4da16a86b9ce33e', 'width': 64}]</t>
   </si>
   <si>
+    <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273c9703979ebcc156cebd0e2c4', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02c9703979ebcc156cebd0e2c4', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851c9703979ebcc156cebd0e2c4', 'width': 64}]</t>
+  </si>
+  <si>
+    <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b2730b0fbaf16e4475ad616b41b8', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e020b0fbaf16e4475ad616b41b8', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d000048510b0fbaf16e4475ad616b41b8', 'width': 64}]</t>
+  </si>
+  <si>
+    <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273442fa4829200552c55a8f45e', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02442fa4829200552c55a8f45e', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851442fa4829200552c55a8f45e', 'width': 64}]</t>
+  </si>
+  <si>
     <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b2739f2023d391c3bd4acf4d51c6', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e029f2023d391c3bd4acf4d51c6', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d000048519f2023d391c3bd4acf4d51c6', 'width': 64}]</t>
   </si>
   <si>
-    <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b2732dd8a31709137799f5c937f2', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e022dd8a31709137799f5c937f2', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d000048512dd8a31709137799f5c937f2', 'width': 64}]</t>
-  </si>
-  <si>
-    <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b2730b0fbaf16e4475ad616b41b8', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e020b0fbaf16e4475ad616b41b8', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d000048510b0fbaf16e4475ad616b41b8', 'width': 64}]</t>
-  </si>
-  <si>
     <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273787674b6a114f98cad6f834b', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02787674b6a114f98cad6f834b', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851787674b6a114f98cad6f834b', 'width': 64}]</t>
   </si>
   <si>
-    <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273c9703979ebcc156cebd0e2c4', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02c9703979ebcc156cebd0e2c4', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851c9703979ebcc156cebd0e2c4', 'width': 64}]</t>
-  </si>
-  <si>
-    <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273442fa4829200552c55a8f45e', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02442fa4829200552c55a8f45e', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851442fa4829200552c55a8f45e', 'width': 64}]</t>
-  </si>
-  <si>
     <t>Scorpion</t>
   </si>
   <si>
@@ -157,21 +157,21 @@
     <t>Love At First Sting</t>
   </si>
   <si>
+    <t>Lovedrive</t>
+  </si>
+  <si>
+    <t>Blackout</t>
+  </si>
+  <si>
+    <t>World Wide Live</t>
+  </si>
+  <si>
     <t>Comeblack</t>
   </si>
   <si>
-    <t>Blackout</t>
-  </si>
-  <si>
     <t>Crazy World</t>
   </si>
   <si>
-    <t>Lovedrive</t>
-  </si>
-  <si>
-    <t>World Wide Live</t>
-  </si>
-  <si>
     <t>2018-06-29</t>
   </si>
   <si>
@@ -181,27 +181,27 @@
     <t>2001-03-06</t>
   </si>
   <si>
+    <t>2001-02-25</t>
+  </si>
+  <si>
     <t>1984-03-27</t>
   </si>
   <si>
+    <t>1979-02-25</t>
+  </si>
+  <si>
+    <t>1982-04-10</t>
+  </si>
+  <si>
+    <t>1985-06-20</t>
+  </si>
+  <si>
     <t>2011-11-07</t>
   </si>
   <si>
-    <t>2001-02-25</t>
-  </si>
-  <si>
-    <t>1982-04-10</t>
-  </si>
-  <si>
     <t>1990-01-01</t>
   </si>
   <si>
-    <t>1979-02-25</t>
-  </si>
-  <si>
-    <t>1985-06-20</t>
-  </si>
-  <si>
     <t>day</t>
   </si>
   <si>
@@ -214,27 +214,27 @@
     <t>spotify:album:6ZWL1xSTEvqs5A6dBh8vZw</t>
   </si>
   <si>
+    <t>spotify:album:2epkTConsXtPOHY9QhvqeR</t>
+  </si>
+  <si>
     <t>spotify:album:71cfSO0iO1fjgQLEb3Wc6C</t>
   </si>
   <si>
+    <t>spotify:album:7aIgGWlHdcPXOfONtXVliK</t>
+  </si>
+  <si>
+    <t>spotify:album:6x75r5C54z1quun86Bbqbr</t>
+  </si>
+  <si>
+    <t>spotify:album:5z5s71RoLOhdB8SwPfru0I</t>
+  </si>
+  <si>
     <t>spotify:album:4vQ96yyyYbaeTQujH3iTtd</t>
   </si>
   <si>
-    <t>spotify:album:2epkTConsXtPOHY9QhvqeR</t>
-  </si>
-  <si>
-    <t>spotify:album:6x75r5C54z1quun86Bbqbr</t>
-  </si>
-  <si>
     <t>spotify:album:3dLKM8bD8R3H3XnSOXGjTF</t>
   </si>
   <si>
-    <t>spotify:album:7aIgGWlHdcPXOfONtXVliK</t>
-  </si>
-  <si>
-    <t>spotify:album:5z5s71RoLOhdB8SwPfru0I</t>
-  </si>
-  <si>
     <t>[{'external_urls': {'spotify': 'https://open.spotify.com/artist/3TVXtAsR1Inumwj472S9r4'}, 'href': 'https://api.spotify.com/v1/artists/3TVXtAsR1Inumwj472S9r4', 'id': '3TVXtAsR1Inumwj472S9r4', 'name': 'Drake', 'type': 'artist', 'uri': 'spotify:artist:3TVXtAsR1Inumwj472S9r4'}]</t>
   </si>
   <si>
@@ -253,25 +253,25 @@
     <t>https://open.spotify.com/album/6ZWL1xSTEvqs5A6dBh8vZw</t>
   </si>
   <si>
+    <t>https://open.spotify.com/album/2epkTConsXtPOHY9QhvqeR</t>
+  </si>
+  <si>
     <t>https://open.spotify.com/album/71cfSO0iO1fjgQLEb3Wc6C</t>
   </si>
   <si>
+    <t>https://open.spotify.com/album/7aIgGWlHdcPXOfONtXVliK</t>
+  </si>
+  <si>
+    <t>https://open.spotify.com/album/6x75r5C54z1quun86Bbqbr</t>
+  </si>
+  <si>
+    <t>https://open.spotify.com/album/5z5s71RoLOhdB8SwPfru0I</t>
+  </si>
+  <si>
     <t>https://open.spotify.com/album/4vQ96yyyYbaeTQujH3iTtd</t>
   </si>
   <si>
-    <t>https://open.spotify.com/album/2epkTConsXtPOHY9QhvqeR</t>
-  </si>
-  <si>
-    <t>https://open.spotify.com/album/6x75r5C54z1quun86Bbqbr</t>
-  </si>
-  <si>
     <t>https://open.spotify.com/album/3dLKM8bD8R3H3XnSOXGjTF</t>
-  </si>
-  <si>
-    <t>https://open.spotify.com/album/7aIgGWlHdcPXOfONtXVliK</t>
-  </si>
-  <si>
-    <t>https://open.spotify.com/album/5z5s71RoLOhdB8SwPfru0I</t>
   </si>
 </sst>
 </file>
@@ -814,7 +814,7 @@
         <v>13</v>
       </c>
       <c r="B5">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="C5" t="b">
         <v>1</v>
@@ -829,7 +829,7 @@
         <v>37</v>
       </c>
       <c r="G5" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="H5" t="s">
         <v>55</v>
@@ -844,7 +844,7 @@
         <v>66</v>
       </c>
       <c r="L5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M5" s="2" t="s">
         <v>79</v>
@@ -855,7 +855,7 @@
         <v>13</v>
       </c>
       <c r="B6">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C6" t="b">
         <v>1</v>
@@ -870,7 +870,7 @@
         <v>38</v>
       </c>
       <c r="G6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H6" t="s">
         <v>56</v>
@@ -896,7 +896,7 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -911,7 +911,7 @@
         <v>39</v>
       </c>
       <c r="G7" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H7" t="s">
         <v>57</v>
@@ -926,7 +926,7 @@
         <v>68</v>
       </c>
       <c r="L7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="M7" s="2" t="s">
         <v>81</v>
@@ -978,7 +978,7 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
@@ -1019,7 +1019,7 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
@@ -1060,7 +1060,7 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
Atualização dos código de teste da biblioteca
</commit_message>
<xml_diff>
--- a/backend/arq/search_albums_scorpion.xlsx
+++ b/backend/arq/search_albums_scorpion.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="87">
   <si>
     <t>album_type</t>
   </si>
@@ -73,9 +73,6 @@
     <t>https://api.spotify.com/v1/albums/71cfSO0iO1fjgQLEb3Wc6C</t>
   </si>
   <si>
-    <t>https://api.spotify.com/v1/albums/7aIgGWlHdcPXOfONtXVliK</t>
-  </si>
-  <si>
     <t>https://api.spotify.com/v1/albums/6x75r5C54z1quun86Bbqbr</t>
   </si>
   <si>
@@ -88,6 +85,9 @@
     <t>https://api.spotify.com/v1/albums/3dLKM8bD8R3H3XnSOXGjTF</t>
   </si>
   <si>
+    <t>https://api.spotify.com/v1/albums/6fgLXQA1I40kOPXy8G4BK8</t>
+  </si>
+  <si>
     <t>1ATL5GLyefJaxhQzSPVrLX</t>
   </si>
   <si>
@@ -103,9 +103,6 @@
     <t>71cfSO0iO1fjgQLEb3Wc6C</t>
   </si>
   <si>
-    <t>7aIgGWlHdcPXOfONtXVliK</t>
-  </si>
-  <si>
     <t>6x75r5C54z1quun86Bbqbr</t>
   </si>
   <si>
@@ -118,6 +115,9 @@
     <t>3dLKM8bD8R3H3XnSOXGjTF</t>
   </si>
   <si>
+    <t>6fgLXQA1I40kOPXy8G4BK8</t>
+  </si>
+  <si>
     <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273f907de96b9a4fbc04accc0d5', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02f907de96b9a4fbc04accc0d5', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851f907de96b9a4fbc04accc0d5', 'width': 64}]</t>
   </si>
   <si>
@@ -133,9 +133,6 @@
     <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273926764eed4da16a86b9ce33e', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02926764eed4da16a86b9ce33e', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851926764eed4da16a86b9ce33e', 'width': 64}]</t>
   </si>
   <si>
-    <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273c9703979ebcc156cebd0e2c4', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02c9703979ebcc156cebd0e2c4', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851c9703979ebcc156cebd0e2c4', 'width': 64}]</t>
-  </si>
-  <si>
     <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b2730b0fbaf16e4475ad616b41b8', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e020b0fbaf16e4475ad616b41b8', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d000048510b0fbaf16e4475ad616b41b8', 'width': 64}]</t>
   </si>
   <si>
@@ -148,6 +145,9 @@
     <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273787674b6a114f98cad6f834b', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02787674b6a114f98cad6f834b', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851787674b6a114f98cad6f834b', 'width': 64}]</t>
   </si>
   <si>
+    <t>[{'height': 640, 'url': 'https://i.scdn.co/image/ab67616d0000b273eb021b18fcead1189954756d', 'width': 640}, {'height': 300, 'url': 'https://i.scdn.co/image/ab67616d00001e02eb021b18fcead1189954756d', 'width': 300}, {'height': 64, 'url': 'https://i.scdn.co/image/ab67616d00004851eb021b18fcead1189954756d', 'width': 64}]</t>
+  </si>
+  <si>
     <t>Scorpion</t>
   </si>
   <si>
@@ -157,9 +157,6 @@
     <t>Love At First Sting</t>
   </si>
   <si>
-    <t>Lovedrive</t>
-  </si>
-  <si>
     <t>Blackout</t>
   </si>
   <si>
@@ -172,6 +169,9 @@
     <t>Crazy World</t>
   </si>
   <si>
+    <t>CAOS</t>
+  </si>
+  <si>
     <t>2018-06-29</t>
   </si>
   <si>
@@ -187,9 +187,6 @@
     <t>1984-03-27</t>
   </si>
   <si>
-    <t>1979-02-25</t>
-  </si>
-  <si>
     <t>1982-04-10</t>
   </si>
   <si>
@@ -202,6 +199,9 @@
     <t>1990-01-01</t>
   </si>
   <si>
+    <t>2024-09-23</t>
+  </si>
+  <si>
     <t>day</t>
   </si>
   <si>
@@ -220,9 +220,6 @@
     <t>spotify:album:71cfSO0iO1fjgQLEb3Wc6C</t>
   </si>
   <si>
-    <t>spotify:album:7aIgGWlHdcPXOfONtXVliK</t>
-  </si>
-  <si>
     <t>spotify:album:6x75r5C54z1quun86Bbqbr</t>
   </si>
   <si>
@@ -235,6 +232,9 @@
     <t>spotify:album:3dLKM8bD8R3H3XnSOXGjTF</t>
   </si>
   <si>
+    <t>spotify:album:6fgLXQA1I40kOPXy8G4BK8</t>
+  </si>
+  <si>
     <t>[{'external_urls': {'spotify': 'https://open.spotify.com/artist/3TVXtAsR1Inumwj472S9r4'}, 'href': 'https://api.spotify.com/v1/artists/3TVXtAsR1Inumwj472S9r4', 'id': '3TVXtAsR1Inumwj472S9r4', 'name': 'Drake', 'type': 'artist', 'uri': 'spotify:artist:3TVXtAsR1Inumwj472S9r4'}]</t>
   </si>
   <si>
@@ -244,6 +244,9 @@
     <t>[{'external_urls': {'spotify': 'https://open.spotify.com/artist/4d3yvTptO48nOYTPBcPFZC'}, 'href': 'https://api.spotify.com/v1/artists/4d3yvTptO48nOYTPBcPFZC', 'id': '4d3yvTptO48nOYTPBcPFZC', 'name': 'Eve', 'type': 'artist', 'uri': 'spotify:artist:4d3yvTptO48nOYTPBcPFZC'}]</t>
   </si>
   <si>
+    <t>[{'external_urls': {'spotify': 'https://open.spotify.com/artist/6rk6Izp6o42fUdE0jRqAP4'}, 'href': 'https://api.spotify.com/v1/artists/6rk6Izp6o42fUdE0jRqAP4', 'id': '6rk6Izp6o42fUdE0jRqAP4', 'name': 'Alee', 'type': 'artist', 'uri': 'spotify:artist:6rk6Izp6o42fUdE0jRqAP4'}]</t>
+  </si>
+  <si>
     <t>https://open.spotify.com/album/1ATL5GLyefJaxhQzSPVrLX</t>
   </si>
   <si>
@@ -259,9 +262,6 @@
     <t>https://open.spotify.com/album/71cfSO0iO1fjgQLEb3Wc6C</t>
   </si>
   <si>
-    <t>https://open.spotify.com/album/7aIgGWlHdcPXOfONtXVliK</t>
-  </si>
-  <si>
     <t>https://open.spotify.com/album/6x75r5C54z1quun86Bbqbr</t>
   </si>
   <si>
@@ -272,6 +272,9 @@
   </si>
   <si>
     <t>https://open.spotify.com/album/3dLKM8bD8R3H3XnSOXGjTF</t>
+  </si>
+  <si>
+    <t>https://open.spotify.com/album/6fgLXQA1I40kOPXy8G4BK8</t>
   </si>
 </sst>
 </file>
@@ -724,7 +727,7 @@
         <v>73</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -765,7 +768,7 @@
         <v>74</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -806,7 +809,7 @@
         <v>75</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -847,7 +850,7 @@
         <v>75</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -888,7 +891,7 @@
         <v>74</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -896,7 +899,7 @@
         <v>13</v>
       </c>
       <c r="B7">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C7" t="b">
         <v>1</v>
@@ -929,7 +932,7 @@
         <v>74</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -937,7 +940,7 @@
         <v>13</v>
       </c>
       <c r="B8">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="C8" t="b">
         <v>1</v>
@@ -970,7 +973,7 @@
         <v>74</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -978,7 +981,7 @@
         <v>13</v>
       </c>
       <c r="B9">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="C9" t="b">
         <v>1</v>
@@ -1011,7 +1014,7 @@
         <v>74</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -1019,7 +1022,7 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C10" t="b">
         <v>1</v>
@@ -1052,7 +1055,7 @@
         <v>74</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1060,7 +1063,7 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C11" t="b">
         <v>1</v>
@@ -1090,10 +1093,10 @@
         <v>72</v>
       </c>
       <c r="L11" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>